<commit_message>
until program approved test case
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{246F9E97-CE38-42E9-84F5-C480DDF1B8A9}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{6D517EEC-1196-4147-A4A7-B1BFC75DAAE0}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -87,6 +87,18 @@
   </si>
   <si>
     <t>Automation test description</t>
+  </si>
+  <si>
+    <t>FocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>KPIsRequired__c</t>
+  </si>
+  <si>
+    <t>IsGoalsRequired__c</t>
   </si>
 </sst>
 </file>
@@ -422,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.90625" bestFit="1" customWidth="1"/>
@@ -485,6 +497,48 @@
       </c>
       <c r="D4" s="3" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prgoram all test cases and happy path completed
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{6D517EEC-1196-4147-A4A7-B1BFC75DAAE0}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{56688E0F-7E93-4522-9E43-9A7E1B28580C}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -44,61 +44,64 @@
     <t>ProgramName__c</t>
   </si>
   <si>
+    <t>Dropdown</t>
+  </si>
+  <si>
+    <t>Type__c</t>
+  </si>
+  <si>
+    <t>Project Grants</t>
+  </si>
+  <si>
+    <t>Lookup</t>
+  </si>
+  <si>
+    <t>PrimaryFundingOrganization__c</t>
+  </si>
+  <si>
+    <t>Research And Innovative Technology Administration</t>
+  </si>
+  <si>
+    <t>Overview</t>
+  </si>
+  <si>
+    <t>Abbreviation__c</t>
+  </si>
+  <si>
+    <t>WebsiteAddress__c</t>
+  </si>
+  <si>
+    <t>http://automate.com</t>
+  </si>
+  <si>
+    <t>Objectives__c</t>
+  </si>
+  <si>
+    <t>RichText</t>
+  </si>
+  <si>
+    <t>Automation test description</t>
+  </si>
+  <si>
+    <t>FocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>KPIsRequired__c</t>
+  </si>
+  <si>
+    <t>IsGoalsRequired__c</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>AuPr</t>
+  </si>
+  <si>
     <t>Automation Program</t>
-  </si>
-  <si>
-    <t>Dropdown</t>
-  </si>
-  <si>
-    <t>Type__c</t>
-  </si>
-  <si>
-    <t>Project Grants</t>
-  </si>
-  <si>
-    <t>Lookup</t>
-  </si>
-  <si>
-    <t>PrimaryFundingOrganization__c</t>
-  </si>
-  <si>
-    <t>Research And Innovative Technology Administration</t>
-  </si>
-  <si>
-    <t>Overview</t>
-  </si>
-  <si>
-    <t>Abbreviation__c</t>
-  </si>
-  <si>
-    <t>AuPr</t>
-  </si>
-  <si>
-    <t>WebsiteAddress__c</t>
-  </si>
-  <si>
-    <t>http://automate.com</t>
-  </si>
-  <si>
-    <t>Objectives__c</t>
-  </si>
-  <si>
-    <t>RichText</t>
-  </si>
-  <si>
-    <t>Automation test description</t>
-  </si>
-  <si>
-    <t>FocusAreaRequired__c</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>KPIsRequired__c</t>
-  </si>
-  <si>
-    <t>IsGoalsRequired__c</t>
   </si>
 </sst>
 </file>
@@ -468,7 +471,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -476,13 +479,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -490,13 +493,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -504,13 +507,13 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -518,13 +521,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -532,13 +535,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -573,44 +576,44 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
         <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Announcement until approved status
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{56688E0F-7E93-4522-9E43-9A7E1B28580C}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{99704BF7-2F35-46A9-8D5E-3B4490928DA6}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -93,9 +93,6 @@
   </si>
   <si>
     <t>IsGoalsRequired__c</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>AuPr</t>
@@ -471,7 +468,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -527,7 +524,7 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -541,7 +538,7 @@
         <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -585,7 +582,7 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updated the program feature scenarios to be independent
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{99704BF7-2F35-46A9-8D5E-3B4490928DA6}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{50A2D09D-EE85-4CA4-A36E-AA09F8E0518A}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="3" r:id="rId1"/>
@@ -95,10 +95,10 @@
     <t>IsGoalsRequired__c</t>
   </si>
   <si>
-    <t>AuPr</t>
-  </si>
-  <si>
     <t>Automation Program</t>
+  </si>
+  <si>
+    <t>AP</t>
   </si>
 </sst>
 </file>
@@ -468,7 +468,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -582,7 +582,7 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added three new test cases to award feature
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{A1CA3C76-A10A-4400-B2A7-38FC765DCB83}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{42D01BF8-1997-40C7-A603-11603953252E}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RequiredForSave" sheetId="3" r:id="rId1"/>
@@ -95,10 +95,10 @@
     <t>IsGoalsRequired__c</t>
   </si>
   <si>
-    <t>APTD</t>
-  </si>
-  <si>
-    <t>Automation Program to be deleted</t>
+    <t>Automation Program Dec10</t>
+  </si>
+  <si>
+    <t>AD10</t>
   </si>
 </sst>
 </file>
@@ -435,15 +435,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,7 +457,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -468,10 +468,10 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -485,7 +485,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -499,7 +499,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -513,7 +513,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -527,7 +527,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -550,14 +550,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA6F275D-7657-4500-825C-5F565736E8FE}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -571,7 +571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -582,10 +582,10 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -599,7 +599,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Updated the consolidated method for Program feature and have worked four new Site Visit Test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="19126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{5A290231-AA61-4D9C-89C9-7E6A4C457033}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{6F709890-6D22-4A03-80EC-69E38A267F95}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -98,7 +98,7 @@
     <t>AD10</t>
   </si>
   <si>
-    <t>District Court</t>
+    <t>Test Automation Organization</t>
   </si>
 </sst>
 </file>
@@ -541,11 +541,8 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" tooltip="District Court" display="https://test7-internal--c.na57.visual.force.com/0010b00002CmKfwAAF" xr:uid="{855A68A3-A67F-4F57-8D11-7EF523E82526}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Test cases of Closeout
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D0834A-CE7E-42FF-886E-3826546489C8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3A0E2F-F594-40DA-890D-C8430D6B61BF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>Test Automation Organization</t>
+  </si>
+  <si>
+    <t>ProgramName__c</t>
+  </si>
+  <si>
+    <t>Automation Program Jan21</t>
   </si>
 </sst>
 </file>
@@ -428,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" bestFit="1" customWidth="1"/>
@@ -451,11 +457,11 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
+      <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -463,10 +469,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>23</v>
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -474,10 +480,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -485,7 +491,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -496,15 +502,26 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
       </c>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{7EE9E90B-967F-44F2-8381-163CD7361D89}"/>
+    <hyperlink ref="C4" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{7EE9E90B-967F-44F2-8381-163CD7361D89}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
updated the test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCB5E0B-9F5F-47CA-814A-C88EA82A979C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6501002D-26E1-4D98-8265-AB57804412A1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -99,7 +99,7 @@
     <t>PREG</t>
   </si>
   <si>
-    <t>Automation Program  Regression</t>
+    <t>Automation Program Regression</t>
   </si>
 </sst>
 </file>

</xml_diff>